<commit_message>
This new Branch is used for BX72 Board
</commit_message>
<xml_diff>
--- a/help/Ent_contant.xlsx
+++ b/help/Ent_contant.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Designs\UDP\MyUDP0310\help\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Designs\UDP\GIT_UDP\help\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46821E0D-9B4C-4399-B333-B88AEC362306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B5A667A-0D45-4C9D-A01C-23DEF53088CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{0A3A1713-A9CC-44BC-ACAC-9E67F131A9F0}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
   <si>
     <t>des_mac</t>
   </si>
@@ -69,9 +69,6 @@
     <t>Ver;IHL;DSCP;ECN</t>
   </si>
   <si>
-    <t>length</t>
-  </si>
-  <si>
     <t>ID</t>
   </si>
   <si>
@@ -135,25 +132,25 @@
     <t>11</t>
   </si>
   <si>
-    <t>b6c8</t>
-  </si>
-  <si>
     <t>4000</t>
   </si>
   <si>
-    <t>4500</t>
-  </si>
-  <si>
-    <t>4011</t>
-  </si>
-  <si>
-    <t>c0a8</t>
-  </si>
-  <si>
-    <t>0180</t>
-  </si>
-  <si>
-    <t>0127</t>
+    <t>Payload size + 28</t>
+  </si>
+  <si>
+    <t>Payload size + 8</t>
+  </si>
+  <si>
+    <t>IPSize</t>
+  </si>
+  <si>
+    <t>IPcheckSum1 = 16'h4500 + IPSize + 16'h0000 + 16'h0000 + 16'h4011;</t>
+  </si>
+  <si>
+    <t>IPcheckSum2 = local_ip[31:16] + local_ip[15:0] + des_ip[31:16] + des_ip[15:0];</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data (0) </t>
   </si>
 </sst>
 </file>
@@ -507,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C68EFFDF-987A-4C09-9CA0-C289D07FFA84}">
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="9" style="1"/>
@@ -516,7 +513,7 @@
     <col min="11" max="11" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -530,7 +527,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -544,7 +541,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -556,7 +553,7 @@
         <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F3" t="s">
         <v>2</v>
@@ -569,20 +566,10 @@
         <v>14</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="L4">
-        <f>28*8</f>
-        <v>224</v>
-      </c>
-      <c r="M4">
-        <f>L4/64</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -590,7 +577,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
         <v>13</v>
@@ -602,7 +589,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -610,26 +597,22 @@
         <v>2</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="G6">
         <v>2</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="L6">
-        <f>HEX2DEC(K6)</f>
-        <v>17664</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+        <v>31</v>
+      </c>
+      <c r="J6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -637,34 +620,19 @@
         <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="K7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L7">
-        <f t="shared" ref="L7:L14" si="0">HEX2DEC(K7)</f>
-        <v>45</v>
-      </c>
-      <c r="M7">
-        <f>SUM($L$6:L7)</f>
-        <v>17709</v>
-      </c>
-      <c r="N7" t="str">
-        <f>DEC2HEX(M7)</f>
-        <v>452D</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -672,10 +640,10 @@
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G8">
         <v>2</v>
@@ -685,25 +653,10 @@
         <v>8</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="L8">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <f>SUM($L$6:L8)</f>
-        <v>17709</v>
-      </c>
-      <c r="N8" t="str">
-        <f t="shared" ref="N8:P15" si="1">DEC2HEX(M8)</f>
-        <v>452D</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -715,245 +668,166 @@
         <v>8</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L9">
-        <f t="shared" si="0"/>
-        <v>16384</v>
-      </c>
-      <c r="M9">
-        <f>SUM($L$6:L9)</f>
-        <v>34093</v>
-      </c>
-      <c r="N9" t="str">
-        <f t="shared" si="1"/>
-        <v>852D</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="K10" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="L10">
-        <f t="shared" si="0"/>
-        <v>16401</v>
-      </c>
-      <c r="M10">
-        <f>SUM($L$6:L10)</f>
-        <v>50494</v>
-      </c>
-      <c r="N10" t="str">
-        <f t="shared" si="1"/>
-        <v>C53E</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11">
-        <v>6</v>
-      </c>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L11">
-        <f t="shared" si="0"/>
-        <v>49320</v>
-      </c>
-      <c r="N11" t="str">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12">
-        <v>4</v>
-      </c>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G12">
         <v>1</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L12">
-        <f t="shared" si="0"/>
-        <v>384</v>
-      </c>
-      <c r="M12">
-        <f>SUM($L$11:L12)</f>
-        <v>49704</v>
-      </c>
-      <c r="N12" t="str">
-        <f t="shared" si="1"/>
-        <v>C228</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="J13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14">
         <v>6</v>
       </c>
-      <c r="F13" t="s">
+      <c r="J14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="F15" t="s">
         <v>19</v>
-      </c>
-      <c r="G13">
-        <v>2</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="L13">
-        <f t="shared" si="0"/>
-        <v>49320</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14">
-        <v>4</v>
-      </c>
-      <c r="C14">
-        <f>SUM(B10:B14)</f>
-        <v>20</v>
-      </c>
-      <c r="F14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14">
-        <v>4</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L14">
-        <f t="shared" si="0"/>
-        <v>295</v>
-      </c>
-      <c r="M14">
-        <f>SUM($L$13:L14)</f>
-        <v>49615</v>
-      </c>
-      <c r="N14" t="str">
-        <f t="shared" si="1"/>
-        <v>C1CF</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="F15" t="s">
-        <v>21</v>
       </c>
       <c r="G15">
         <v>4</v>
       </c>
-      <c r="H15">
-        <f>SUM(G11:G15)</f>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16">
+        <v>6</v>
+      </c>
+      <c r="F16" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16">
+        <v>4</v>
+      </c>
+      <c r="H16">
+        <f>SUM(G11:G16)</f>
         <v>12</v>
       </c>
-      <c r="M15">
-        <f>SUM(M12:M14)</f>
-        <v>99319</v>
-      </c>
-      <c r="N15" t="str">
-        <f t="shared" si="1"/>
-        <v>183F7</v>
-      </c>
-      <c r="O15">
-        <f>M15+M10</f>
-        <v>149813</v>
-      </c>
-      <c r="P15" t="str">
-        <f t="shared" si="1"/>
-        <v>24935</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="F17" t="s">
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17">
+        <v>4</v>
+      </c>
+      <c r="C17">
+        <f>SUM(B13:B17)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F19" t="s">
         <v>22</v>
       </c>
-      <c r="G17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C18">
+      <c r="G19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F20" t="s">
+        <v>23</v>
+      </c>
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="J20" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F21" t="s">
+        <v>24</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H23">
         <v>18</v>
       </c>
-      <c r="F18" t="s">
-        <v>23</v>
-      </c>
-      <c r="G18">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C19">
-        <f>SUM(C1:C18)</f>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C25">
+        <f>SUM(C1:C24)</f>
         <v>60</v>
       </c>
-      <c r="F19" t="s">
-        <v>24</v>
-      </c>
-      <c r="G19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="F20" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20">
-        <v>2</v>
-      </c>
-      <c r="H20">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H26">
+        <f>SUM(H3:H25)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>12</v>
       </c>
-      <c r="B21">
+      <c r="B27">
         <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H22">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H25">
-        <f>SUM(H3:H24)</f>
-        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
working ARP & UDP packets loopback
</commit_message>
<xml_diff>
--- a/help/Ent_contant.xlsx
+++ b/help/Ent_contant.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Designs\UDP\GIT_UDP\help\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Designs\UDP\MyUDP2510\help\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B5A667A-0D45-4C9D-A01C-23DEF53088CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4978D11-3F5C-48B4-A384-1D70CEC08009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{0A3A1713-A9CC-44BC-ACAC-9E67F131A9F0}"/>
+    <workbookView xWindow="-28905" yWindow="75" windowWidth="14610" windowHeight="15585" xr2:uid="{0A3A1713-A9CC-44BC-ACAC-9E67F131A9F0}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="43">
   <si>
     <t>des_mac</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t xml:space="preserve">Data (0) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">data </t>
   </si>
 </sst>
 </file>
@@ -504,44 +507,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C68EFFDF-987A-4C09-9CA0-C289D07FFA84}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="9" style="1"/>
-    <col min="6" max="6" width="17.375" customWidth="1"/>
-    <col min="9" max="9" width="9" style="1"/>
-    <col min="11" max="11" width="9" style="1"/>
+    <col min="6" max="6" width="9" style="1"/>
+    <col min="8" max="8" width="17.375" customWidth="1"/>
+    <col min="12" max="12" width="9" style="1"/>
+    <col min="14" max="14" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1">
         <v>6</v>
       </c>
-      <c r="F1" t="s">
+      <c r="D1" t="str">
+        <f>DEC2HEX(C1)</f>
         <v>0</v>
       </c>
-      <c r="G1">
+      <c r="H1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K1" t="str">
+        <f>DEC2HEX(J1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2">
         <v>6</v>
       </c>
-      <c r="F2" t="s">
+      <c r="C2">
+        <f>SUM($B$1:B2)</f>
+        <v>12</v>
+      </c>
+      <c r="D2" t="str">
+        <f t="shared" ref="D2:D29" si="0">DEC2HEX(C2)</f>
+        <v>C</v>
+      </c>
+      <c r="H2" t="s">
         <v>1</v>
       </c>
-      <c r="G2">
+      <c r="I2">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J2">
+        <f>SUM($I$1:I2)</f>
+        <v>12</v>
+      </c>
+      <c r="K2" t="str">
+        <f t="shared" ref="K2:K29" si="1">DEC2HEX(J2)</f>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -549,114 +576,191 @@
         <v>2</v>
       </c>
       <c r="C3">
+        <f>SUM($B$1:B3)</f>
+        <v>14</v>
+      </c>
+      <c r="D3" t="str">
+        <f t="shared" si="0"/>
+        <v>E</v>
+      </c>
+      <c r="E3">
         <f>SUM(B1:B3)</f>
         <v>14</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <f>SUM(G1:G3)</f>
+      <c r="H3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <f>SUM($I$1:I3)</f>
         <v>14</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="K3" t="str">
+        <f t="shared" si="1"/>
+        <v>E</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C4">
+        <f>SUM($B$1:B4)</f>
+        <v>14</v>
+      </c>
+      <c r="D4" t="str">
+        <f t="shared" si="0"/>
+        <v>E</v>
+      </c>
+      <c r="J4">
+        <f>SUM($I$1:I4)</f>
+        <v>14</v>
+      </c>
+      <c r="K4" t="str">
+        <f t="shared" si="1"/>
+        <v>E</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5">
         <v>2</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="C5">
+        <f>SUM($B$1:B5)</f>
+        <v>16</v>
+      </c>
+      <c r="D5" t="str">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>13</v>
       </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="I5" s="1">
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L5" s="1">
         <v>4500</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6">
         <v>2</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="C6">
+        <f>SUM($B$1:B6)</f>
+        <v>18</v>
+      </c>
+      <c r="D6" t="str">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>38</v>
       </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <f>SUM($I$6:I6)-1</f>
+        <v>1</v>
+      </c>
+      <c r="K6" t="str">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="L6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J6" t="s">
+      <c r="M6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="C7">
+        <f>SUM($B$1:B7)</f>
+        <v>19</v>
+      </c>
+      <c r="D7" t="str">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>14</v>
       </c>
-      <c r="G7">
-        <v>2</v>
-      </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <f>SUM($I$6:I7)-1</f>
+        <v>3</v>
+      </c>
+      <c r="K7" t="str">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="L7" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="C8">
+        <f>SUM($B$1:B8)</f>
+        <v>20</v>
+      </c>
+      <c r="D8" t="str">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8">
-        <v>2</v>
-      </c>
-      <c r="H8">
-        <f>SUM(G5:G8)</f>
-        <v>8</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J8">
+        <f>SUM($I$6:I8)-1</f>
+        <v>3</v>
+      </c>
+      <c r="K8" t="str">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -664,170 +768,536 @@
         <v>2</v>
       </c>
       <c r="C9">
+        <f>SUM($B$1:B9)</f>
+        <v>22</v>
+      </c>
+      <c r="D9" t="str">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="E9">
         <f>SUM(B5:B9)</f>
         <v>8</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F11" t="s">
+      <c r="H9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9">
+        <v>2</v>
+      </c>
+      <c r="J9">
+        <f>SUM($I$6:I9)-1</f>
+        <v>5</v>
+      </c>
+      <c r="K9" t="str">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C10">
+        <f>SUM($B$1:B10)</f>
+        <v>22</v>
+      </c>
+      <c r="D10" t="str">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="G11">
+      <c r="J10">
+        <f>SUM($I$6:I10)-1</f>
+        <v>5</v>
+      </c>
+      <c r="K10" t="str">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C11">
+        <f>SUM($B$1:B11)</f>
+        <v>22</v>
+      </c>
+      <c r="D11" t="str">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="J11">
+        <f>SUM($I$6:I11)-1</f>
+        <v>5</v>
+      </c>
+      <c r="K11" t="str">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12">
+        <v>6</v>
+      </c>
+      <c r="C12">
+        <f>SUM($B$1:B12)</f>
+        <v>28</v>
+      </c>
+      <c r="D12" t="str">
+        <f t="shared" si="0"/>
+        <v>1C</v>
+      </c>
+      <c r="F12" t="s">
         <v>1</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="H12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <f>SUM($I$6:I12)-1</f>
+        <v>6</v>
+      </c>
+      <c r="K12" t="str">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="L12" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F12" t="s">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C13">
+        <f>SUM($B$1:B13)</f>
+        <v>28</v>
+      </c>
+      <c r="D13" t="str">
+        <f t="shared" si="0"/>
+        <v>1C</v>
+      </c>
+      <c r="H13" t="s">
         <v>17</v>
       </c>
-      <c r="G12">
+      <c r="I13">
         <v>1</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J13">
+        <f>SUM($I$6:I13)-1</f>
+        <v>7</v>
+      </c>
+      <c r="K13" t="str">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="L13" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F13" t="s">
+      <c r="M13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C14">
+        <f>SUM($B$1:B14)</f>
+        <v>28</v>
+      </c>
+      <c r="D14" t="str">
+        <f t="shared" si="0"/>
+        <v>1C</v>
+      </c>
+      <c r="H14" t="s">
         <v>18</v>
       </c>
-      <c r="G13">
-        <v>2</v>
-      </c>
-      <c r="J13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14">
+      <c r="I14">
+        <v>2</v>
+      </c>
+      <c r="J14">
+        <f>SUM($I$6:I14)-1</f>
+        <v>9</v>
+      </c>
+      <c r="K14" t="str">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="M14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C15">
+        <f>SUM($B$1:B15)</f>
+        <v>28</v>
+      </c>
+      <c r="D15" t="str">
+        <f t="shared" si="0"/>
+        <v>1C</v>
+      </c>
+      <c r="J15">
+        <f>SUM($I$6:I15)-1</f>
+        <v>9</v>
+      </c>
+      <c r="K15" t="str">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16">
+        <v>4</v>
+      </c>
+      <c r="C16">
+        <f>SUM($B$1:B16)</f>
+        <v>32</v>
+      </c>
+      <c r="D16" t="str">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="F16" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" t="s">
+        <v>19</v>
+      </c>
+      <c r="I16">
+        <v>4</v>
+      </c>
+      <c r="J16">
+        <f>SUM($I$6:I16)-1</f>
+        <v>13</v>
+      </c>
+      <c r="K16" t="str">
+        <f t="shared" si="1"/>
+        <v>D</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17">
         <v>6</v>
       </c>
-      <c r="J14" t="s">
+      <c r="C17">
+        <f>SUM($B$1:B17)</f>
+        <v>38</v>
+      </c>
+      <c r="D17" t="str">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>0</v>
+      </c>
+      <c r="H17" t="s">
+        <v>20</v>
+      </c>
+      <c r="I17">
+        <v>4</v>
+      </c>
+      <c r="J17">
+        <f>SUM($I$6:I17)-1</f>
+        <v>17</v>
+      </c>
+      <c r="K17" t="str">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <f>SUM($B$1:B18)</f>
+        <v>42</v>
+      </c>
+      <c r="D18" t="str">
+        <f t="shared" si="0"/>
+        <v>2A</v>
+      </c>
+      <c r="E18">
+        <f>SUM(B12:B18)</f>
+        <v>20</v>
+      </c>
+      <c r="F18" t="s">
+        <v>20</v>
+      </c>
+      <c r="J18">
+        <f>SUM($I$6:I18)-1</f>
+        <v>17</v>
+      </c>
+      <c r="K18" t="str">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C19">
+        <f>SUM($B$1:B19)</f>
+        <v>42</v>
+      </c>
+      <c r="D19" t="str">
+        <f t="shared" si="0"/>
+        <v>2A</v>
+      </c>
+      <c r="H19" t="s">
+        <v>21</v>
+      </c>
+      <c r="I19">
+        <v>2</v>
+      </c>
+      <c r="J19">
+        <f>SUM($I$6:I19)-1</f>
+        <v>19</v>
+      </c>
+      <c r="K19" t="str">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C20">
+        <f>SUM($B$1:B20)</f>
+        <v>42</v>
+      </c>
+      <c r="D20" t="str">
+        <f t="shared" si="0"/>
+        <v>2A</v>
+      </c>
+      <c r="H20" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20">
+        <v>2</v>
+      </c>
+      <c r="J20">
+        <f>SUM($I$6:I20)-1</f>
+        <v>21</v>
+      </c>
+      <c r="K20" t="str">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="M20" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C21">
+        <f>SUM($B$1:B21)</f>
+        <v>42</v>
+      </c>
+      <c r="D21" t="str">
+        <f t="shared" si="0"/>
+        <v>2A</v>
+      </c>
+      <c r="H21" t="s">
+        <v>23</v>
+      </c>
+      <c r="I21">
+        <v>2</v>
+      </c>
+      <c r="J21">
+        <f>SUM($I$6:I21)-1</f>
+        <v>23</v>
+      </c>
+      <c r="K21" t="str">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C22">
+        <f>SUM($B$1:B22)</f>
+        <v>42</v>
+      </c>
+      <c r="D22" t="str">
+        <f t="shared" si="0"/>
+        <v>2A</v>
+      </c>
+      <c r="H22" t="s">
+        <v>24</v>
+      </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
+      <c r="J22">
+        <f>SUM($I$6:I22)-1</f>
+        <v>25</v>
+      </c>
+      <c r="K22" t="str">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C23">
+        <f>SUM($B$1:B23)</f>
+        <v>42</v>
+      </c>
+      <c r="D23" t="str">
+        <f t="shared" si="0"/>
+        <v>2A</v>
+      </c>
+      <c r="J23">
+        <f>SUM($I$6:I23)-1</f>
+        <v>25</v>
+      </c>
+      <c r="K23" t="str">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C24">
+        <f>SUM($B$1:B24)</f>
+        <v>42</v>
+      </c>
+      <c r="D24" t="str">
+        <f t="shared" si="0"/>
+        <v>2A</v>
+      </c>
+      <c r="J24">
+        <f>SUM($I$6:I24)-1</f>
+        <v>25</v>
+      </c>
+      <c r="K24" t="str">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25">
+        <v>18</v>
+      </c>
+      <c r="C25">
+        <f>SUM($B$1:B25)</f>
+        <v>60</v>
+      </c>
+      <c r="D25" t="str">
+        <f t="shared" si="0"/>
+        <v>3C</v>
+      </c>
+      <c r="E25">
+        <v>18</v>
+      </c>
+      <c r="H25" t="s">
+        <v>42</v>
+      </c>
+      <c r="I25">
+        <v>18</v>
+      </c>
+      <c r="J25">
+        <f>SUM($I$6:I25)-1</f>
+        <v>43</v>
+      </c>
+      <c r="K25" t="str">
+        <f t="shared" si="1"/>
+        <v>2B</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C26">
+        <f>SUM($B$1:B26)</f>
+        <v>60</v>
+      </c>
+      <c r="D26" t="str">
+        <f t="shared" si="0"/>
+        <v>3C</v>
+      </c>
+      <c r="E26">
+        <f>SUM(E1:E25)</f>
+        <v>60</v>
+      </c>
+      <c r="J26">
+        <f>SUM($I$6:I26)-1</f>
+        <v>43</v>
+      </c>
+      <c r="K26" t="str">
+        <f t="shared" si="1"/>
+        <v>2B</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C27">
+        <f>SUM($B$1:B27)</f>
+        <v>60</v>
+      </c>
+      <c r="D27" t="str">
+        <f t="shared" si="0"/>
+        <v>3C</v>
+      </c>
+      <c r="J27">
+        <f>SUM($I$6:I27)-1</f>
+        <v>43</v>
+      </c>
+      <c r="K27" t="str">
+        <f t="shared" si="1"/>
+        <v>2B</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28">
+        <v>4</v>
+      </c>
+      <c r="C28">
+        <f>SUM($B$1:B28)</f>
+        <v>64</v>
+      </c>
+      <c r="D28" t="str">
+        <f t="shared" si="0"/>
         <v>40</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15">
+      <c r="H28" t="s">
+        <v>12</v>
+      </c>
+      <c r="I28">
         <v>4</v>
       </c>
-      <c r="F15" t="s">
-        <v>19</v>
-      </c>
-      <c r="G15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16">
-        <v>6</v>
-      </c>
-      <c r="F16" t="s">
-        <v>20</v>
-      </c>
-      <c r="G16">
-        <v>4</v>
-      </c>
-      <c r="H16">
-        <f>SUM(G11:G16)</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17">
-        <v>4</v>
-      </c>
-      <c r="C17">
-        <f>SUM(B13:B17)</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F18" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F19" t="s">
-        <v>22</v>
-      </c>
-      <c r="G19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F20" t="s">
-        <v>23</v>
-      </c>
-      <c r="G20">
-        <v>2</v>
-      </c>
-      <c r="J20" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="F21" t="s">
-        <v>24</v>
-      </c>
-      <c r="G21">
-        <v>2</v>
-      </c>
-      <c r="H21">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="H23">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="C25">
-        <f>SUM(C1:C24)</f>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="H26">
-        <f>SUM(H3:H25)</f>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>12</v>
-      </c>
-      <c r="B27">
-        <v>4</v>
+      <c r="J28">
+        <f>SUM($I$6:I28)-1</f>
+        <v>47</v>
+      </c>
+      <c r="K28" t="str">
+        <f t="shared" si="1"/>
+        <v>2F</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="C29">
+        <f>SUM($B$1:B29)</f>
+        <v>64</v>
+      </c>
+      <c r="D29" t="str">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+      <c r="J29">
+        <f>SUM($I$6:I29)-1</f>
+        <v>47</v>
+      </c>
+      <c r="K29" t="str">
+        <f t="shared" si="1"/>
+        <v>2F</v>
       </c>
     </row>
   </sheetData>

</xml_diff>